<commit_message>
feat: add SEO bulk fields and category pricing
</commit_message>
<xml_diff>
--- a/public/samples/sarjan-product-bulk-upload-sample.xlsx
+++ b/public/samples/sarjan-product-bulk-upload-sample.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:W3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,42 +407,66 @@
         <v>sku</v>
       </c>
       <c r="C1" t="str">
+        <v>category_level_1</v>
+      </c>
+      <c r="D1" t="str">
+        <v>category_level_2</v>
+      </c>
+      <c r="E1" t="str">
+        <v>category_level_3</v>
+      </c>
+      <c r="F1" t="str">
+        <v>category_path</v>
+      </c>
+      <c r="G1" t="str">
         <v>category</v>
       </c>
-      <c r="D1" t="str">
+      <c r="H1" t="str">
         <v>fabric</v>
       </c>
-      <c r="E1" t="str">
+      <c r="I1" t="str">
         <v>price</v>
       </c>
-      <c r="F1" t="str">
+      <c r="J1" t="str">
         <v>moq</v>
       </c>
-      <c r="G1" t="str">
+      <c r="K1" t="str">
         <v>stock</v>
       </c>
-      <c r="H1" t="str">
+      <c r="L1" t="str">
         <v>reserved</v>
       </c>
-      <c r="I1" t="str">
+      <c r="M1" t="str">
         <v>sold</v>
       </c>
-      <c r="J1" t="str">
+      <c r="N1" t="str">
         <v>colors</v>
       </c>
-      <c r="K1" t="str">
+      <c r="O1" t="str">
         <v>sizes</v>
       </c>
-      <c r="L1" t="str">
+      <c r="P1" t="str">
         <v>description</v>
       </c>
-      <c r="M1" t="str">
+      <c r="Q1" t="str">
         <v>care</v>
       </c>
-      <c r="N1" t="str">
+      <c r="R1" t="str">
         <v>image_urls</v>
       </c>
-      <c r="O1" t="str">
+      <c r="S1" t="str">
+        <v>image_alt</v>
+      </c>
+      <c r="T1" t="str">
+        <v>meta_title</v>
+      </c>
+      <c r="U1" t="str">
+        <v>meta_description</v>
+      </c>
+      <c r="V1" t="str">
+        <v>keywords</v>
+      </c>
+      <c r="W1" t="str">
         <v>is_featured</v>
       </c>
     </row>
@@ -454,42 +478,66 @@
         <v>SAR-SH-AJ-IND</v>
       </c>
       <c r="C2" t="str">
+        <v>Men</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Shirts</v>
+      </c>
+      <c r="E2" t="str">
         <v>Printed Shirts</v>
       </c>
-      <c r="D2" t="str">
+      <c r="F2" t="str">
+        <v>Men, Shirts, Printed Shirts</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Printed Shirts</v>
+      </c>
+      <c r="H2" t="str">
         <v>Cotton cambric</v>
       </c>
-      <c r="E2">
+      <c r="I2">
         <v>680</v>
       </c>
-      <c r="F2">
+      <c r="J2">
         <v>24</v>
       </c>
-      <c r="G2">
+      <c r="K2">
         <v>420</v>
       </c>
-      <c r="H2">
+      <c r="L2">
         <v>0</v>
       </c>
-      <c r="I2">
+      <c r="M2">
         <v>0</v>
       </c>
-      <c r="J2" t="str">
+      <c r="N2" t="str">
         <v>Indigo, Black, Ivory</v>
       </c>
-      <c r="K2" t="str">
+      <c r="O2" t="str">
         <v>S, M, L, XL</v>
       </c>
-      <c r="L2" t="str">
+      <c r="P2" t="str">
         <v>Wholesale-ready Ajrak inspired printed shirt.</v>
       </c>
-      <c r="M2" t="str">
+      <c r="Q2" t="str">
         <v>Gentle wash separately. Dry in shade.</v>
       </c>
-      <c r="N2" t="str">
+      <c r="R2" t="str">
         <v>/sarjan-assets/shirt-ajrak-black-studio.png</v>
       </c>
-      <c r="O2" t="str">
+      <c r="S2" t="str">
+        <v>Ajrak indigo printed shirt for wholesale buyers</v>
+      </c>
+      <c r="T2" t="str">
+        <v>Ajrak Indigo Shirt for Wholesale Buyers</v>
+      </c>
+      <c r="U2" t="str">
+        <v>Buy Ajrak Indigo Shirt in B2B wholesale size runs with cotton cambric fabric, MOQ planning, and ready stock from Sarjan Textiles.</v>
+      </c>
+      <c r="V2" t="str">
+        <v>ajrak shirt, indigo printed shirt, wholesale shirt, cotton cambric</v>
+      </c>
+      <c r="W2" t="str">
         <v>yes</v>
       </c>
     </row>
@@ -498,51 +546,75 @@
         <v>Blue Floral Kurta</v>
       </c>
       <c r="B3" t="str">
-        <v>SAR-KU-BL-FLR-NEW</v>
+        <v>SAR-KU-BL-FLR</v>
       </c>
       <c r="C3" t="str">
+        <v>Men</v>
+      </c>
+      <c r="D3" t="str">
         <v>Kurtas</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
+        <v>Floral Kurtas</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Men, Kurtas, Floral Kurtas</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Floral Kurtas</v>
+      </c>
+      <c r="H3" t="str">
         <v>Rayon cotton blend</v>
       </c>
-      <c r="E3">
+      <c r="I3">
         <v>820</v>
       </c>
-      <c r="F3">
+      <c r="J3">
         <v>18</v>
       </c>
-      <c r="G3">
+      <c r="K3">
         <v>260</v>
       </c>
-      <c r="H3">
+      <c r="L3">
         <v>0</v>
       </c>
-      <c r="I3">
+      <c r="M3">
         <v>0</v>
       </c>
-      <c r="J3" t="str">
+      <c r="N3" t="str">
         <v>Blue, Peach, Teal</v>
       </c>
-      <c r="K3" t="str">
+      <c r="O3" t="str">
         <v>M, L, XL, XXL</v>
       </c>
-      <c r="L3" t="str">
-        <v>Soft floral kurta range for repeat B2B orders.</v>
-      </c>
-      <c r="M3" t="str">
-        <v>Hand wash recommended.</v>
-      </c>
-      <c r="N3" t="str">
+      <c r="P3" t="str">
+        <v>Soft floral kurta range for retail-ready festive assortments.</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>Hand wash recommended. Iron inside out.</v>
+      </c>
+      <c r="R3" t="str">
         <v>/sarjan-assets/kurta-blue-floral-studio.png</v>
       </c>
-      <c r="O3" t="str">
-        <v>no</v>
+      <c r="S3" t="str">
+        <v>Blue floral kurta wholesale product image</v>
+      </c>
+      <c r="T3" t="str">
+        <v>Blue Floral Kurta Wholesale Collection</v>
+      </c>
+      <c r="U3" t="str">
+        <v>Explore Blue Floral Kurta wholesale collection with rayon cotton blend fabric, color variants, MOQ, and B2B ordering support.</v>
+      </c>
+      <c r="V3" t="str">
+        <v>blue floral kurta, wholesale kurta, rayon cotton kurta</v>
+      </c>
+      <c r="W3" t="str">
+        <v>yes</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Treat bulk and admin stock as full set counts per size group.
stock_regular and stock_plus now mean available sets per color (not per-piece), with an updated sample sheet and set-aware availability on the storefront.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/samples/sarjan-product-bulk-upload-sample.xlsx
+++ b/public/samples/sarjan-product-bulk-upload-sample.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="39">
   <si>
     <t>name</t>
   </si>
@@ -35,9 +35,6 @@
     <t>sizes_plus</t>
   </si>
   <si>
-    <t>stock_by_size</t>
-  </si>
-  <si>
     <t>stock_regular</t>
   </si>
   <si>
@@ -53,9 +50,6 @@
     <t>moq</t>
   </si>
   <si>
-    <t>stock</t>
-  </si>
-  <si>
     <t>description</t>
   </si>
   <si>
@@ -89,13 +83,10 @@
     <t>3XL,4XL,5XL</t>
   </si>
   <si>
-    <t>S:20|M:25|L:30|XL:20|XXL:15|3XL:10|4XL:8|5XL:5</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
-    <t>Sample bulk row. Customer can order XS-XXL set or 3XL-5XL set separately.</t>
+    <t>Sample row: 10 regular sets + 5 plus sets per color. Customer qty 3 = 3 full sets.</t>
   </si>
   <si>
     <t>Gentle wash separately, Dry in shade</t>
@@ -110,34 +101,34 @@
     <t>Example</t>
   </si>
   <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>XS to XXL group. Optional if sizes column has all sizes.</t>
-  </si>
-  <si>
-    <t>Plus group up to 5XL only (no Free Size).</t>
-  </si>
-  <si>
-    <t>S:20|M:25|3XL:10</t>
-  </si>
-  <si>
-    <t>Same piece qty for every color. Use | or , between sizes.</t>
-  </si>
-  <si>
-    <t>stock_regular / stock_plus</t>
-  </si>
-  <si>
-    <t>20 / 8</t>
-  </si>
-  <si>
-    <t>Same qty per size in that group for all colors.</t>
-  </si>
-  <si>
-    <t>Indigo:S:20,Maroon:3XL:8</t>
-  </si>
-  <si>
-    <t>Per color+size pieces. Overrides stock_by_size for those cells.</t>
+    <t>Meaning</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>10 full sets per color for XS–XXL group. 1 set = one piece of each size in sizes_regular.</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>5 full sets per color for 3XL–5XL group.</t>
+  </si>
+  <si>
+    <t>Customer order qty</t>
+  </si>
+  <si>
+    <t>3 sets</t>
+  </si>
+  <si>
+    <t>3 complete sets — not 3 individual pieces.</t>
+  </si>
+  <si>
+    <t>Indigo:S:12,Maroon:3XL:6</t>
+  </si>
+  <si>
+    <t>Optional per-color override (values are still SET count).</t>
   </si>
 </sst>
 </file>
@@ -524,19 +515,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="17" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="9" width="17" customWidth="1"/>
-    <col min="10" max="10" width="16" customWidth="1"/>
-    <col min="11" max="11" width="17" customWidth="1"/>
-    <col min="12" max="18" width="16" customWidth="1"/>
+    <col min="1" max="16" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -585,67 +570,55 @@
       <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="B2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="C2" t="s">
         <v>18</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>19</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>20</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>21</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
         <v>22</v>
       </c>
-      <c r="F2" t="s">
+      <c r="H2">
+        <v>10</v>
+      </c>
+      <c r="I2">
+        <v>5</v>
+      </c>
+      <c r="J2" t="s">
         <v>23</v>
       </c>
-      <c r="G2" t="s">
+      <c r="K2">
+        <v>120</v>
+      </c>
+      <c r="L2">
+        <v>12</v>
+      </c>
+      <c r="M2" t="s">
         <v>24</v>
       </c>
-      <c r="H2" t="s">
+      <c r="N2" t="s">
         <v>25</v>
       </c>
-      <c r="I2" t="s">
+      <c r="O2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P2" t="s">
         <v>26</v>
-      </c>
-      <c r="J2" t="s">
-        <v>26</v>
-      </c>
-      <c r="K2" t="s">
-        <v>26</v>
-      </c>
-      <c r="L2">
-        <v>120</v>
-      </c>
-      <c r="M2">
-        <v>12</v>
-      </c>
-      <c r="N2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>26</v>
-      </c>
-      <c r="R2" t="s">
-        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -656,50 +629,50 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="52" customWidth="1"/>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="56" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>34</v>
       </c>
       <c r="B4" t="s">
         <v>35</v>
@@ -710,24 +683,13 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
         <v>37</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>38</v>
-      </c>
-      <c r="C5" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C6" t="s">
-        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>